<commit_message>
more results 9 - dim red + feat sel + agressive oversampling
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\uni\MEI 1ano1sem\DAA\trabalho\DAA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54769D0E-843A-4EB0-85CC-EA843817E8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22213A50-5106-428B-8CA5-533593317BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="14020" xr2:uid="{744B1543-7C44-49C5-883E-AA14D96B6E1A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="281">
   <si>
     <t>DAA tests and results</t>
   </si>
@@ -719,21 +719,6 @@
     <t>LightGBM1</t>
   </si>
   <si>
-    <t>None of the models provide super stable results, but some are interesting</t>
-  </si>
-  <si>
-    <t>Next step is to perfom more agressive oversampling</t>
-  </si>
-  <si>
-    <t>Fifth batch of tests - Oversampling without Dimensionality</t>
-  </si>
-  <si>
-    <t>Considering the last batche's results weren't completely inconsistent,</t>
-  </si>
-  <si>
-    <t>It's probably worth it to test na agressive way of oversampling again.</t>
-  </si>
-  <si>
     <t>In this batch, data treatment is the same as in the fourth besides for the oversampling.</t>
   </si>
   <si>
@@ -798,6 +783,102 @@
   </si>
   <si>
     <t>0.311</t>
+  </si>
+  <si>
+    <t>0.351</t>
+  </si>
+  <si>
+    <t>Considering the last batch's results weren't completely inconsistent,</t>
+  </si>
+  <si>
+    <t>It's probably worth it to test an agressive way of oversampling again.</t>
+  </si>
+  <si>
+    <t>majority class</t>
+  </si>
+  <si>
+    <t>Fifth batch of tests - Agressive oversampling without Dimensionality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reduction and feature selection. We did this because the results obtained at batch 3 are </t>
+  </si>
+  <si>
+    <t>too inconsistent. We want to confirm if it is normal or there was any error while measuring</t>
+  </si>
+  <si>
+    <t>them</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;None of the models provide super stable results, but some are interesting</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;Next step is to perfom more agressive oversampling</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;These models don't provide stable results either</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;While it might seem counter-productive, the next step is to test this with dimensionality</t>
+  </si>
+  <si>
+    <t>Sixth batch of tests - Agressive oversampling with Dimensionality</t>
+  </si>
+  <si>
+    <t>As explained in the fifth batch's conclusions part, we want to double check the</t>
+  </si>
+  <si>
+    <t>results obtained on the third batch.</t>
+  </si>
+  <si>
+    <t>We are using last batch's oversampling paramethers (class2 by 0.33 of majority class</t>
+  </si>
+  <si>
+    <t>and all others by 1.0 of majority class). Nothing changed on the data treatment part,</t>
+  </si>
+  <si>
+    <t>besides for adding dimensionality reduction and feature selection.</t>
+  </si>
+  <si>
+    <t>ANOVA (200)</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>PCA (100)</t>
+  </si>
+  <si>
+    <t>0.474</t>
+  </si>
+  <si>
+    <t>0.604</t>
+  </si>
+  <si>
+    <t>0.368</t>
+  </si>
+  <si>
+    <t>0.450</t>
+  </si>
+  <si>
+    <t>0.574</t>
+  </si>
+  <si>
+    <t>0.572</t>
+  </si>
+  <si>
+    <t>0.545</t>
+  </si>
+  <si>
+    <t>0.569</t>
+  </si>
+  <si>
+    <t>dimensionality reduction and feature selection description</t>
+  </si>
+  <si>
+    <t>0.28</t>
+  </si>
+  <si>
+    <t>0.380</t>
   </si>
 </sst>
 </file>
@@ -882,7 +963,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -1286,11 +1367,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1516,8 +1612,20 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1525,25 +1633,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1564,21 +1663,23 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1882,14 +1983,16 @@
   <dimension ref="A1:BU476"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.90625" customWidth="1"/>
-    <col min="10" max="10" width="17.08984375" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" customWidth="1"/>
+    <col min="10" max="10" width="17.1796875" customWidth="1"/>
     <col min="18" max="18" width="19.1796875" customWidth="1"/>
     <col min="25" max="25" width="8.7265625" customWidth="1"/>
-    <col min="26" max="26" width="16.90625" customWidth="1"/>
+    <col min="26" max="26" width="16.81640625" customWidth="1"/>
     <col min="27" max="27" width="73.7265625" customWidth="1"/>
     <col min="33" max="33" width="23.453125" customWidth="1"/>
     <col min="35" max="35" width="18.1796875" customWidth="1"/>
+    <col min="41" max="41" width="49.54296875" customWidth="1"/>
+    <col min="43" max="43" width="15.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:73" x14ac:dyDescent="0.35">
@@ -2066,16 +2169,16 @@
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="89" t="s">
+      <c r="R3" s="109" t="s">
         <v>119</v>
       </c>
-      <c r="S3" s="89"/>
-      <c r="T3" s="89"/>
-      <c r="U3" s="89"/>
-      <c r="V3" s="89"/>
-      <c r="W3" s="89"/>
-      <c r="X3" s="89"/>
-      <c r="Y3" s="89"/>
+      <c r="S3" s="109"/>
+      <c r="T3" s="109"/>
+      <c r="U3" s="109"/>
+      <c r="V3" s="109"/>
+      <c r="W3" s="109"/>
+      <c r="X3" s="109"/>
+      <c r="Y3" s="109"/>
       <c r="Z3" s="73" t="s">
         <v>149</v>
       </c>
@@ -2086,7 +2189,7 @@
       <c r="AE3" s="73"/>
       <c r="AF3" s="73"/>
       <c r="AG3" s="73" t="s">
-        <v>229</v>
+        <v>253</v>
       </c>
       <c r="AH3" s="73"/>
       <c r="AI3" s="1"/>
@@ -2095,8 +2198,10 @@
       <c r="AL3" s="1"/>
       <c r="AM3" s="1"/>
       <c r="AN3" s="1"/>
-      <c r="AO3" s="1"/>
-      <c r="AP3" s="1"/>
+      <c r="AO3" s="73" t="s">
+        <v>261</v>
+      </c>
+      <c r="AP3" s="73"/>
       <c r="AQ3" s="1"/>
       <c r="AR3" s="1"/>
       <c r="AS3" s="1"/>
@@ -2129,7 +2234,7 @@
       <c r="BT3" s="1"/>
       <c r="BU3" s="1"/>
     </row>
-    <row r="4" spans="1:73" ht="15.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:73" ht="15.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1"/>
       <c r="B4" s="4" t="s">
         <v>47</v>
@@ -2151,16 +2256,16 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
-      <c r="R4" s="89" t="s">
+      <c r="R4" s="109" t="s">
         <v>120</v>
       </c>
-      <c r="S4" s="89"/>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="89"/>
-      <c r="W4" s="89"/>
-      <c r="X4" s="89"/>
-      <c r="Y4" s="89"/>
+      <c r="S4" s="109"/>
+      <c r="T4" s="109"/>
+      <c r="U4" s="109"/>
+      <c r="V4" s="109"/>
+      <c r="W4" s="109"/>
+      <c r="X4" s="109"/>
+      <c r="Y4" s="109"/>
       <c r="Z4" s="73" t="s">
         <v>150</v>
       </c>
@@ -2180,8 +2285,10 @@
       <c r="AL4" s="1"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="1"/>
-      <c r="AO4" s="1"/>
-      <c r="AP4" s="1"/>
+      <c r="AO4" s="73" t="s">
+        <v>150</v>
+      </c>
+      <c r="AP4" s="73"/>
       <c r="AQ4" s="1"/>
       <c r="AR4" s="1"/>
       <c r="AS4" s="1"/>
@@ -2254,7 +2361,7 @@
       <c r="AE5" s="1"/>
       <c r="AF5" s="1"/>
       <c r="AG5" s="4" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="AH5" s="1"/>
       <c r="AI5" s="1"/>
@@ -2263,7 +2370,9 @@
       <c r="AL5" s="1"/>
       <c r="AM5" s="1"/>
       <c r="AN5" s="1"/>
-      <c r="AO5" s="1"/>
+      <c r="AO5" s="4" t="s">
+        <v>262</v>
+      </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="1"/>
       <c r="AR5" s="1"/>
@@ -2347,7 +2456,7 @@
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
@@ -2356,7 +2465,9 @@
       <c r="AL6" s="1"/>
       <c r="AM6" s="1"/>
       <c r="AN6" s="1"/>
-      <c r="AO6" s="1"/>
+      <c r="AO6" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="1"/>
       <c r="AR6" s="1"/>
@@ -2436,7 +2547,7 @@
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="AH7" s="1"/>
       <c r="AI7" s="1"/>
@@ -2445,7 +2556,9 @@
       <c r="AL7" s="1"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="1"/>
-      <c r="AO7" s="1"/>
+      <c r="AO7" s="1" t="s">
+        <v>264</v>
+      </c>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="1"/>
       <c r="AR7" s="1"/>
@@ -2529,7 +2642,7 @@
       <c r="AE8" s="1"/>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="AH8" s="1"/>
       <c r="AI8" s="1"/>
@@ -2538,7 +2651,9 @@
       <c r="AL8" s="1"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="1"/>
-      <c r="AO8" s="1"/>
+      <c r="AO8" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="1"/>
       <c r="AR8" s="1"/>
@@ -2616,7 +2731,7 @@
       <c r="AE9" s="1"/>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="AH9" s="1"/>
       <c r="AI9" s="1"/>
@@ -2625,7 +2740,9 @@
       <c r="AL9" s="1"/>
       <c r="AM9" s="1"/>
       <c r="AN9" s="1"/>
-      <c r="AO9" s="1"/>
+      <c r="AO9" s="1" t="s">
+        <v>266</v>
+      </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="1"/>
       <c r="AR9" s="1"/>
@@ -2833,11 +2950,21 @@
       <c r="AL11" s="1"/>
       <c r="AM11" s="1"/>
       <c r="AN11" s="1"/>
-      <c r="AO11" s="1"/>
-      <c r="AP11" s="1"/>
-      <c r="AQ11" s="1"/>
-      <c r="AR11" s="1"/>
-      <c r="AS11" s="1"/>
+      <c r="AO11" s="110" t="s">
+        <v>278</v>
+      </c>
+      <c r="AP11" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ11" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="AR11" s="59" t="s">
+        <v>2</v>
+      </c>
+      <c r="AS11" s="47" t="s">
+        <v>3</v>
+      </c>
       <c r="AT11" s="1"/>
       <c r="AU11" s="1"/>
       <c r="AV11" s="1"/>
@@ -2927,22 +3054,28 @@
       <c r="AG12" s="7"/>
       <c r="AH12" s="69"/>
       <c r="AI12" s="50" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AJ12" s="50" t="s">
+        <v>241</v>
+      </c>
+      <c r="AK12" s="20" t="s">
         <v>246</v>
-      </c>
-      <c r="AK12" s="20" t="s">
-        <v>251</v>
       </c>
       <c r="AL12" s="1"/>
       <c r="AM12" s="1"/>
       <c r="AN12" s="1"/>
-      <c r="AO12" s="1"/>
-      <c r="AP12" s="1"/>
-      <c r="AQ12" s="1"/>
-      <c r="AR12" s="1"/>
-      <c r="AS12" s="1"/>
+      <c r="AO12" s="8"/>
+      <c r="AP12" s="51"/>
+      <c r="AQ12" s="57" t="s">
+        <v>220</v>
+      </c>
+      <c r="AR12" s="60" t="s">
+        <v>270</v>
+      </c>
+      <c r="AS12" s="20" t="s">
+        <v>279</v>
+      </c>
       <c r="AT12" s="1"/>
       <c r="AU12" s="1"/>
       <c r="AV12" s="1"/>
@@ -3030,14 +3163,14 @@
       <c r="AE13" s="1"/>
       <c r="AF13" s="1"/>
       <c r="AG13" s="8" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AH13" s="51"/>
       <c r="AI13" s="57" t="s">
         <v>222</v>
       </c>
       <c r="AJ13" s="57" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="AK13" s="20" t="s">
         <v>213</v>
@@ -3045,11 +3178,17 @@
       <c r="AL13" s="1"/>
       <c r="AM13" s="1"/>
       <c r="AN13" s="1"/>
-      <c r="AO13" s="1"/>
-      <c r="AP13" s="1"/>
-      <c r="AQ13" s="1"/>
-      <c r="AR13" s="1"/>
-      <c r="AS13" s="1"/>
+      <c r="AO13" s="8"/>
+      <c r="AP13" s="51"/>
+      <c r="AQ13" s="57" t="s">
+        <v>222</v>
+      </c>
+      <c r="AR13" s="60" t="s">
+        <v>28</v>
+      </c>
+      <c r="AS13" s="20" t="s">
+        <v>280</v>
+      </c>
       <c r="AT13" s="1"/>
       <c r="AU13" s="1"/>
       <c r="AV13" s="1"/>
@@ -3141,7 +3280,7 @@
       <c r="AE14" s="1"/>
       <c r="AF14" s="1"/>
       <c r="AG14" s="8" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="AH14" s="51" t="s">
         <v>16</v>
@@ -3150,19 +3289,23 @@
         <v>224</v>
       </c>
       <c r="AJ14" s="88" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="AK14" s="20" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="AL14" s="1"/>
       <c r="AM14" s="1"/>
       <c r="AN14" s="1"/>
-      <c r="AO14" s="1"/>
-      <c r="AP14" s="1"/>
-      <c r="AQ14" s="1"/>
-      <c r="AR14" s="1"/>
-      <c r="AS14" s="1"/>
+      <c r="AO14" s="8"/>
+      <c r="AP14" s="51"/>
+      <c r="AQ14" s="57" t="s">
+        <v>224</v>
+      </c>
+      <c r="AR14" s="61" t="s">
+        <v>271</v>
+      </c>
+      <c r="AS14" s="20"/>
       <c r="AT14" s="1"/>
       <c r="AU14" s="1"/>
       <c r="AV14" s="1"/>
@@ -3260,26 +3403,32 @@
       <c r="AE15" s="1"/>
       <c r="AF15" s="1"/>
       <c r="AG15" s="8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="AH15" s="51"/>
       <c r="AI15" s="52" t="s">
         <v>225</v>
       </c>
       <c r="AJ15" s="52" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="AK15" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="AL15" s="1"/>
       <c r="AM15" s="1"/>
       <c r="AN15" s="1"/>
-      <c r="AO15" s="1"/>
-      <c r="AP15" s="1"/>
-      <c r="AQ15" s="1"/>
-      <c r="AR15" s="1"/>
-      <c r="AS15" s="1"/>
+      <c r="AO15" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="AP15" s="51"/>
+      <c r="AQ15" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="AR15" s="62" t="s">
+        <v>272</v>
+      </c>
+      <c r="AS15" s="42"/>
       <c r="AT15" s="1"/>
       <c r="AU15" s="1"/>
       <c r="AV15" s="1"/>
@@ -3359,40 +3508,50 @@
       <c r="W16" s="1"/>
       <c r="X16" s="1"/>
       <c r="Y16" s="1"/>
-      <c r="Z16" s="90" t="s">
+      <c r="Z16" s="94" t="s">
         <v>218</v>
       </c>
       <c r="AA16" s="78" t="s">
         <v>161</v>
       </c>
-      <c r="AB16" s="92" t="s">
+      <c r="AB16" s="89" t="s">
         <v>163</v>
       </c>
-      <c r="AC16" s="94" t="s">
+      <c r="AC16" s="91" t="s">
         <v>103</v>
       </c>
       <c r="AD16" s="1"/>
       <c r="AE16" s="1"/>
       <c r="AF16" s="1"/>
-      <c r="AG16" s="74"/>
+      <c r="AG16" s="74" t="s">
+        <v>252</v>
+      </c>
       <c r="AH16" s="72"/>
       <c r="AI16" s="58" t="s">
         <v>226</v>
       </c>
       <c r="AJ16" s="58" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="AK16" s="44" t="s">
-        <v>29</v>
+        <v>249</v>
       </c>
       <c r="AL16" s="1"/>
       <c r="AM16" s="1"/>
       <c r="AN16" s="1"/>
-      <c r="AO16" s="1"/>
-      <c r="AP16" s="1"/>
-      <c r="AQ16" s="1"/>
-      <c r="AR16" s="1"/>
-      <c r="AS16" s="1"/>
+      <c r="AO16" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="AP16" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ16" s="52" t="s">
+        <v>226</v>
+      </c>
+      <c r="AR16" s="62" t="s">
+        <v>273</v>
+      </c>
+      <c r="AS16" s="42"/>
       <c r="AT16" s="1"/>
       <c r="AU16" s="1"/>
       <c r="AV16" s="1"/>
@@ -3470,12 +3629,12 @@
       <c r="W17" s="1"/>
       <c r="X17" s="1"/>
       <c r="Y17" s="1"/>
-      <c r="Z17" s="90"/>
+      <c r="Z17" s="94"/>
       <c r="AA17" s="78" t="s">
         <v>165</v>
       </c>
-      <c r="AB17" s="92"/>
-      <c r="AC17" s="94"/>
+      <c r="AB17" s="89"/>
+      <c r="AC17" s="91"/>
       <c r="AD17" s="1"/>
       <c r="AE17" s="1"/>
       <c r="AF17" s="1"/>
@@ -3487,11 +3646,17 @@
       <c r="AL17" s="1"/>
       <c r="AM17" s="1"/>
       <c r="AN17" s="1"/>
-      <c r="AO17" s="1"/>
-      <c r="AP17" s="1"/>
-      <c r="AQ17" s="1"/>
-      <c r="AR17" s="1"/>
-      <c r="AS17" s="1"/>
+      <c r="AO17" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="AP17" s="52"/>
+      <c r="AQ17" s="52" t="s">
+        <v>234</v>
+      </c>
+      <c r="AR17" s="62" t="s">
+        <v>274</v>
+      </c>
+      <c r="AS17" s="42"/>
       <c r="AT17" s="1"/>
       <c r="AU17" s="1"/>
       <c r="AV17" s="1"/>
@@ -3521,7 +3686,7 @@
       <c r="BT17" s="1"/>
       <c r="BU17" s="1"/>
     </row>
-    <row r="18" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:73" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="25" t="s">
         <v>57</v>
@@ -3567,16 +3732,18 @@
       <c r="W18" s="1"/>
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
-      <c r="Z18" s="91"/>
+      <c r="Z18" s="95"/>
       <c r="AA18" s="79" t="s">
         <v>162</v>
       </c>
-      <c r="AB18" s="93"/>
-      <c r="AC18" s="95"/>
+      <c r="AB18" s="97"/>
+      <c r="AC18" s="99"/>
       <c r="AD18" s="1"/>
       <c r="AE18" s="1"/>
       <c r="AF18" s="1"/>
-      <c r="AG18" s="87"/>
+      <c r="AG18" s="13" t="s">
+        <v>73</v>
+      </c>
       <c r="AH18" s="87"/>
       <c r="AI18" s="1"/>
       <c r="AJ18" s="1"/>
@@ -3584,11 +3751,15 @@
       <c r="AL18" s="1"/>
       <c r="AM18" s="1"/>
       <c r="AN18" s="1"/>
-      <c r="AO18" s="1"/>
-      <c r="AP18" s="1"/>
-      <c r="AQ18" s="1"/>
-      <c r="AR18" s="1"/>
-      <c r="AS18" s="1"/>
+      <c r="AO18" s="111"/>
+      <c r="AP18" s="52"/>
+      <c r="AQ18" s="52" t="s">
+        <v>236</v>
+      </c>
+      <c r="AR18" s="62" t="s">
+        <v>275</v>
+      </c>
+      <c r="AS18" s="42"/>
       <c r="AT18" s="1"/>
       <c r="AU18" s="1"/>
       <c r="AV18" s="1"/>
@@ -3666,22 +3837,24 @@
       <c r="W19" s="1"/>
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
-      <c r="Z19" s="96" t="s">
+      <c r="Z19" s="106" t="s">
         <v>219</v>
       </c>
       <c r="AA19" s="82" t="s">
         <v>161</v>
       </c>
-      <c r="AB19" s="99" t="s">
+      <c r="AB19" s="100" t="s">
         <v>117</v>
       </c>
-      <c r="AC19" s="102" t="s">
+      <c r="AC19" s="103" t="s">
         <v>166</v>
       </c>
       <c r="AD19" s="1"/>
       <c r="AE19" s="1"/>
       <c r="AF19" s="1"/>
-      <c r="AG19" s="1"/>
+      <c r="AG19" s="1" t="s">
+        <v>259</v>
+      </c>
       <c r="AH19" s="1"/>
       <c r="AI19" s="1"/>
       <c r="AJ19" s="1"/>
@@ -3689,11 +3862,15 @@
       <c r="AL19" s="1"/>
       <c r="AM19" s="1"/>
       <c r="AN19" s="1"/>
-      <c r="AO19" s="1"/>
-      <c r="AP19" s="1"/>
-      <c r="AQ19" s="1"/>
-      <c r="AR19" s="1"/>
-      <c r="AS19" s="1"/>
+      <c r="AO19" s="111"/>
+      <c r="AP19" s="52"/>
+      <c r="AQ19" s="52" t="s">
+        <v>239</v>
+      </c>
+      <c r="AR19" s="62" t="s">
+        <v>276</v>
+      </c>
+      <c r="AS19" s="42"/>
       <c r="AT19" s="1"/>
       <c r="AU19" s="1"/>
       <c r="AV19" s="1"/>
@@ -3723,7 +3900,7 @@
       <c r="BT19" s="1"/>
       <c r="BU19" s="1"/>
     </row>
-    <row r="20" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:73" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
       <c r="B20" s="19" t="s">
         <v>56</v>
@@ -3775,16 +3952,18 @@
       <c r="W20" s="1"/>
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
-      <c r="Z20" s="97"/>
+      <c r="Z20" s="107"/>
       <c r="AA20" s="84" t="s">
         <v>164</v>
       </c>
-      <c r="AB20" s="100"/>
-      <c r="AC20" s="103"/>
+      <c r="AB20" s="101"/>
+      <c r="AC20" s="104"/>
       <c r="AD20" s="1"/>
       <c r="AE20" s="1"/>
       <c r="AF20" s="1"/>
-      <c r="AG20" s="1"/>
+      <c r="AG20" s="1" t="s">
+        <v>260</v>
+      </c>
       <c r="AH20" s="1"/>
       <c r="AI20" s="1"/>
       <c r="AJ20" s="1"/>
@@ -3792,11 +3971,15 @@
       <c r="AL20" s="1"/>
       <c r="AM20" s="1"/>
       <c r="AN20" s="1"/>
-      <c r="AO20" s="1"/>
-      <c r="AP20" s="1"/>
-      <c r="AQ20" s="1"/>
-      <c r="AR20" s="1"/>
-      <c r="AS20" s="1"/>
+      <c r="AO20" s="112"/>
+      <c r="AP20" s="58"/>
+      <c r="AQ20" s="58" t="s">
+        <v>240</v>
+      </c>
+      <c r="AR20" s="68" t="s">
+        <v>277</v>
+      </c>
+      <c r="AS20" s="44"/>
       <c r="AT20" s="1"/>
       <c r="AU20" s="1"/>
       <c r="AV20" s="1"/>
@@ -3878,16 +4061,18 @@
       <c r="W21" s="1"/>
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
-      <c r="Z21" s="98"/>
+      <c r="Z21" s="108"/>
       <c r="AA21" s="86" t="s">
         <v>162</v>
       </c>
-      <c r="AB21" s="101"/>
-      <c r="AC21" s="104"/>
+      <c r="AB21" s="102"/>
+      <c r="AC21" s="105"/>
       <c r="AD21" s="1"/>
       <c r="AE21" s="1"/>
       <c r="AF21" s="1"/>
-      <c r="AG21" s="1"/>
+      <c r="AG21" s="1" t="s">
+        <v>254</v>
+      </c>
       <c r="AH21" s="1"/>
       <c r="AI21" s="1"/>
       <c r="AJ21" s="1"/>
@@ -3981,22 +4166,24 @@
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
-      <c r="Z22" s="105" t="s">
+      <c r="Z22" s="93" t="s">
         <v>220</v>
       </c>
       <c r="AA22" s="80" t="s">
         <v>215</v>
       </c>
-      <c r="AB22" s="106" t="s">
+      <c r="AB22" s="96" t="s">
         <v>214</v>
       </c>
-      <c r="AC22" s="107" t="s">
+      <c r="AC22" s="98" t="s">
         <v>217</v>
       </c>
       <c r="AD22" s="1"/>
       <c r="AE22" s="1"/>
       <c r="AF22" s="1"/>
-      <c r="AG22" s="1"/>
+      <c r="AG22" s="1" t="s">
+        <v>255</v>
+      </c>
       <c r="AH22" s="1"/>
       <c r="AI22" s="1"/>
       <c r="AJ22" s="1"/>
@@ -4090,16 +4277,18 @@
       <c r="W23" s="1"/>
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
-      <c r="Z23" s="90"/>
+      <c r="Z23" s="94"/>
       <c r="AA23" s="78" t="s">
         <v>216</v>
       </c>
-      <c r="AB23" s="92"/>
-      <c r="AC23" s="94"/>
+      <c r="AB23" s="89"/>
+      <c r="AC23" s="91"/>
       <c r="AD23" s="1"/>
       <c r="AE23" s="1"/>
       <c r="AF23" s="1"/>
-      <c r="AG23" s="1"/>
+      <c r="AG23" s="1" t="s">
+        <v>256</v>
+      </c>
       <c r="AH23" s="1"/>
       <c r="AI23" s="1"/>
       <c r="AJ23" s="1"/>
@@ -4187,12 +4376,12 @@
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
       <c r="Y24" s="1"/>
-      <c r="Z24" s="91"/>
+      <c r="Z24" s="95"/>
       <c r="AA24" s="79" t="s">
         <v>162</v>
       </c>
-      <c r="AB24" s="93"/>
-      <c r="AC24" s="95"/>
+      <c r="AB24" s="97"/>
+      <c r="AC24" s="99"/>
       <c r="AD24" s="1"/>
       <c r="AE24" s="1"/>
       <c r="AF24" s="1"/>
@@ -4282,16 +4471,16 @@
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
-      <c r="Z25" s="96" t="s">
+      <c r="Z25" s="106" t="s">
         <v>221</v>
       </c>
       <c r="AA25" s="82" t="s">
         <v>169</v>
       </c>
-      <c r="AB25" s="99" t="s">
+      <c r="AB25" s="100" t="s">
         <v>193</v>
       </c>
-      <c r="AC25" s="102" t="s">
+      <c r="AC25" s="103" t="s">
         <v>204</v>
       </c>
       <c r="AD25" s="1"/>
@@ -4383,12 +4572,12 @@
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
-      <c r="Z26" s="97"/>
+      <c r="Z26" s="107"/>
       <c r="AA26" s="84" t="s">
         <v>167</v>
       </c>
-      <c r="AB26" s="100"/>
-      <c r="AC26" s="103"/>
+      <c r="AB26" s="101"/>
+      <c r="AC26" s="104"/>
       <c r="AD26" s="1"/>
       <c r="AE26" s="1"/>
       <c r="AF26" s="1"/>
@@ -4476,12 +4665,12 @@
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
-      <c r="Z27" s="98"/>
+      <c r="Z27" s="108"/>
       <c r="AA27" s="86" t="s">
         <v>168</v>
       </c>
-      <c r="AB27" s="101"/>
-      <c r="AC27" s="104"/>
+      <c r="AB27" s="102"/>
+      <c r="AC27" s="105"/>
       <c r="AD27" s="1"/>
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
@@ -4571,16 +4760,16 @@
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
-      <c r="Z28" s="105" t="s">
+      <c r="Z28" s="93" t="s">
         <v>222</v>
       </c>
       <c r="AA28" s="80" t="s">
         <v>169</v>
       </c>
-      <c r="AB28" s="106" t="s">
+      <c r="AB28" s="96" t="s">
         <v>194</v>
       </c>
-      <c r="AC28" s="107" t="s">
+      <c r="AC28" s="98" t="s">
         <v>205</v>
       </c>
       <c r="AD28" s="1"/>
@@ -4674,12 +4863,12 @@
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
-      <c r="Z29" s="90"/>
+      <c r="Z29" s="94"/>
       <c r="AA29" s="78" t="s">
         <v>170</v>
       </c>
-      <c r="AB29" s="92"/>
-      <c r="AC29" s="94"/>
+      <c r="AB29" s="89"/>
+      <c r="AC29" s="91"/>
       <c r="AD29" s="1"/>
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
@@ -4767,12 +4956,12 @@
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
-      <c r="Z30" s="91"/>
+      <c r="Z30" s="95"/>
       <c r="AA30" s="79" t="s">
         <v>168</v>
       </c>
-      <c r="AB30" s="93"/>
-      <c r="AC30" s="95"/>
+      <c r="AB30" s="97"/>
+      <c r="AC30" s="99"/>
       <c r="AD30" s="1"/>
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
@@ -4858,16 +5047,16 @@
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
-      <c r="Z31" s="96" t="s">
+      <c r="Z31" s="106" t="s">
         <v>223</v>
       </c>
       <c r="AA31" s="82" t="s">
         <v>174</v>
       </c>
-      <c r="AB31" s="99" t="s">
+      <c r="AB31" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="AC31" s="102" t="s">
+      <c r="AC31" s="103" t="s">
         <v>10</v>
       </c>
       <c r="AD31" s="1"/>
@@ -4951,12 +5140,12 @@
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>
       <c r="Y32" s="1"/>
-      <c r="Z32" s="97"/>
+      <c r="Z32" s="107"/>
       <c r="AA32" s="84" t="s">
         <v>175</v>
       </c>
-      <c r="AB32" s="100"/>
-      <c r="AC32" s="103"/>
+      <c r="AB32" s="101"/>
+      <c r="AC32" s="104"/>
       <c r="AD32" s="1"/>
       <c r="AE32" s="1"/>
       <c r="AF32" s="1"/>
@@ -5038,12 +5227,12 @@
       <c r="W33" s="1"/>
       <c r="X33" s="1"/>
       <c r="Y33" s="1"/>
-      <c r="Z33" s="98"/>
+      <c r="Z33" s="108"/>
       <c r="AA33" s="86" t="s">
         <v>173</v>
       </c>
-      <c r="AB33" s="101"/>
-      <c r="AC33" s="104"/>
+      <c r="AB33" s="102"/>
+      <c r="AC33" s="105"/>
       <c r="AD33" s="1"/>
       <c r="AE33" s="1"/>
       <c r="AF33" s="1"/>
@@ -5123,16 +5312,16 @@
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
       <c r="Y34" s="1"/>
-      <c r="Z34" s="105" t="s">
+      <c r="Z34" s="93" t="s">
         <v>224</v>
       </c>
       <c r="AA34" s="80" t="s">
         <v>171</v>
       </c>
-      <c r="AB34" s="106" t="s">
+      <c r="AB34" s="96" t="s">
         <v>195</v>
       </c>
-      <c r="AC34" s="107" t="s">
+      <c r="AC34" s="98" t="s">
         <v>102</v>
       </c>
       <c r="AD34" s="1"/>
@@ -5216,12 +5405,12 @@
       <c r="W35" s="1"/>
       <c r="X35" s="1"/>
       <c r="Y35" s="1"/>
-      <c r="Z35" s="90"/>
+      <c r="Z35" s="94"/>
       <c r="AA35" s="78" t="s">
         <v>172</v>
       </c>
-      <c r="AB35" s="92"/>
-      <c r="AC35" s="94"/>
+      <c r="AB35" s="89"/>
+      <c r="AC35" s="91"/>
       <c r="AD35" s="1"/>
       <c r="AE35" s="1"/>
       <c r="AF35" s="1"/>
@@ -5299,12 +5488,12 @@
       <c r="W36" s="1"/>
       <c r="X36" s="1"/>
       <c r="Y36" s="1"/>
-      <c r="Z36" s="91"/>
+      <c r="Z36" s="95"/>
       <c r="AA36" s="79" t="s">
         <v>173</v>
       </c>
-      <c r="AB36" s="93"/>
-      <c r="AC36" s="95"/>
+      <c r="AB36" s="97"/>
+      <c r="AC36" s="99"/>
       <c r="AD36" s="1"/>
       <c r="AE36" s="1"/>
       <c r="AF36" s="1"/>
@@ -5384,16 +5573,16 @@
       <c r="W37" s="1"/>
       <c r="X37" s="1"/>
       <c r="Y37" s="1"/>
-      <c r="Z37" s="96" t="s">
+      <c r="Z37" s="106" t="s">
         <v>225</v>
       </c>
       <c r="AA37" s="82" t="s">
         <v>176</v>
       </c>
-      <c r="AB37" s="99" t="s">
+      <c r="AB37" s="100" t="s">
         <v>196</v>
       </c>
-      <c r="AC37" s="102" t="s">
+      <c r="AC37" s="103" t="s">
         <v>206</v>
       </c>
       <c r="AD37" s="1"/>
@@ -5477,12 +5666,12 @@
       <c r="W38" s="1"/>
       <c r="X38" s="1"/>
       <c r="Y38" s="1"/>
-      <c r="Z38" s="97"/>
+      <c r="Z38" s="107"/>
       <c r="AA38" s="84" t="s">
         <v>177</v>
       </c>
-      <c r="AB38" s="100"/>
-      <c r="AC38" s="103"/>
+      <c r="AB38" s="101"/>
+      <c r="AC38" s="104"/>
       <c r="AD38" s="1"/>
       <c r="AE38" s="1"/>
       <c r="AF38" s="1"/>
@@ -5562,12 +5751,12 @@
       <c r="W39" s="1"/>
       <c r="X39" s="1"/>
       <c r="Y39" s="1"/>
-      <c r="Z39" s="98"/>
+      <c r="Z39" s="108"/>
       <c r="AA39" s="86" t="s">
         <v>178</v>
       </c>
-      <c r="AB39" s="101"/>
-      <c r="AC39" s="104"/>
+      <c r="AB39" s="102"/>
+      <c r="AC39" s="105"/>
       <c r="AD39" s="1"/>
       <c r="AE39" s="1"/>
       <c r="AF39" s="1"/>
@@ -5647,16 +5836,16 @@
       <c r="W40" s="1"/>
       <c r="X40" s="1"/>
       <c r="Y40" s="1"/>
-      <c r="Z40" s="105" t="s">
+      <c r="Z40" s="93" t="s">
         <v>226</v>
       </c>
       <c r="AA40" s="80" t="s">
         <v>179</v>
       </c>
-      <c r="AB40" s="106" t="s">
+      <c r="AB40" s="96" t="s">
         <v>197</v>
       </c>
-      <c r="AC40" s="107" t="s">
+      <c r="AC40" s="98" t="s">
         <v>207</v>
       </c>
       <c r="AD40" s="1"/>
@@ -5740,12 +5929,12 @@
       <c r="W41" s="1"/>
       <c r="X41" s="1"/>
       <c r="Y41" s="1"/>
-      <c r="Z41" s="90"/>
+      <c r="Z41" s="94"/>
       <c r="AA41" s="78" t="s">
         <v>180</v>
       </c>
-      <c r="AB41" s="92"/>
-      <c r="AC41" s="94"/>
+      <c r="AB41" s="89"/>
+      <c r="AC41" s="91"/>
       <c r="AD41" s="1"/>
       <c r="AE41" s="1"/>
       <c r="AF41" s="1"/>
@@ -5825,12 +6014,12 @@
       <c r="W42" s="1"/>
       <c r="X42" s="1"/>
       <c r="Y42" s="1"/>
-      <c r="Z42" s="91"/>
+      <c r="Z42" s="95"/>
       <c r="AA42" s="79" t="s">
         <v>181</v>
       </c>
-      <c r="AB42" s="93"/>
-      <c r="AC42" s="95"/>
+      <c r="AB42" s="97"/>
+      <c r="AC42" s="99"/>
       <c r="AD42" s="1"/>
       <c r="AE42" s="1"/>
       <c r="AF42" s="1"/>
@@ -5903,15 +6092,15 @@
       <c r="X43" s="1"/>
       <c r="Y43" s="1"/>
       <c r="Z43" s="83" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="AA43" s="82" t="s">
         <v>183</v>
       </c>
-      <c r="AB43" s="99" t="s">
+      <c r="AB43" s="100" t="s">
         <v>198</v>
       </c>
-      <c r="AC43" s="102" t="s">
+      <c r="AC43" s="103" t="s">
         <v>208</v>
       </c>
       <c r="AD43" s="1"/>
@@ -5993,8 +6182,8 @@
       <c r="AA44" s="84" t="s">
         <v>184</v>
       </c>
-      <c r="AB44" s="100"/>
-      <c r="AC44" s="103"/>
+      <c r="AB44" s="101"/>
+      <c r="AC44" s="104"/>
       <c r="AD44" s="1"/>
       <c r="AE44" s="1"/>
       <c r="AF44" s="1"/>
@@ -6072,8 +6261,8 @@
       <c r="AA45" s="86" t="s">
         <v>185</v>
       </c>
-      <c r="AB45" s="101"/>
-      <c r="AC45" s="104"/>
+      <c r="AB45" s="102"/>
+      <c r="AC45" s="105"/>
       <c r="AD45" s="1"/>
       <c r="AE45" s="1"/>
       <c r="AF45" s="1"/>
@@ -6148,15 +6337,15 @@
       <c r="X46" s="1"/>
       <c r="Y46" s="1"/>
       <c r="Z46" s="75" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="AA46" s="80" t="s">
         <v>186</v>
       </c>
-      <c r="AB46" s="106" t="s">
+      <c r="AB46" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="AC46" s="107" t="s">
+      <c r="AC46" s="98" t="s">
         <v>209</v>
       </c>
       <c r="AD46" s="1"/>
@@ -6238,8 +6427,8 @@
       <c r="AA47" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="AB47" s="92"/>
-      <c r="AC47" s="94"/>
+      <c r="AB47" s="89"/>
+      <c r="AC47" s="91"/>
       <c r="AD47" s="1"/>
       <c r="AE47" s="1"/>
       <c r="AF47" s="1"/>
@@ -6317,8 +6506,8 @@
       <c r="AA48" s="79" t="s">
         <v>185</v>
       </c>
-      <c r="AB48" s="93"/>
-      <c r="AC48" s="95"/>
+      <c r="AB48" s="97"/>
+      <c r="AC48" s="99"/>
       <c r="AD48" s="1"/>
       <c r="AE48" s="1"/>
       <c r="AF48" s="1"/>
@@ -6391,15 +6580,15 @@
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
       <c r="Z49" s="83" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="AA49" s="82" t="s">
         <v>187</v>
       </c>
-      <c r="AB49" s="99" t="s">
+      <c r="AB49" s="100" t="s">
         <v>28</v>
       </c>
-      <c r="AC49" s="102" t="s">
+      <c r="AC49" s="103" t="s">
         <v>210</v>
       </c>
       <c r="AD49" s="1"/>
@@ -6479,8 +6668,8 @@
       <c r="AA50" s="84" t="s">
         <v>184</v>
       </c>
-      <c r="AB50" s="100"/>
-      <c r="AC50" s="103"/>
+      <c r="AB50" s="101"/>
+      <c r="AC50" s="104"/>
       <c r="AD50" s="1"/>
       <c r="AE50" s="1"/>
       <c r="AF50" s="1"/>
@@ -6556,8 +6745,8 @@
       <c r="AA51" s="86" t="s">
         <v>185</v>
       </c>
-      <c r="AB51" s="101"/>
-      <c r="AC51" s="104"/>
+      <c r="AB51" s="102"/>
+      <c r="AC51" s="105"/>
       <c r="AD51" s="1"/>
       <c r="AE51" s="1"/>
       <c r="AF51" s="1"/>
@@ -6630,15 +6819,15 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
       <c r="Z52" s="75" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="AA52" s="80" t="s">
         <v>188</v>
       </c>
-      <c r="AB52" s="106" t="s">
+      <c r="AB52" s="96" t="s">
         <v>199</v>
       </c>
-      <c r="AC52" s="107" t="s">
+      <c r="AC52" s="98" t="s">
         <v>211</v>
       </c>
       <c r="AD52" s="1"/>
@@ -6718,8 +6907,8 @@
       <c r="AA53" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="AB53" s="92"/>
-      <c r="AC53" s="94"/>
+      <c r="AB53" s="89"/>
+      <c r="AC53" s="91"/>
       <c r="AD53" s="1"/>
       <c r="AE53" s="1"/>
       <c r="AF53" s="1"/>
@@ -6795,8 +6984,8 @@
       <c r="AA54" s="79" t="s">
         <v>185</v>
       </c>
-      <c r="AB54" s="93"/>
-      <c r="AC54" s="95"/>
+      <c r="AB54" s="97"/>
+      <c r="AC54" s="99"/>
       <c r="AD54" s="1"/>
       <c r="AE54" s="1"/>
       <c r="AF54" s="1"/>
@@ -6869,15 +7058,15 @@
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
       <c r="Z55" s="83" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AA55" s="82" t="s">
         <v>189</v>
       </c>
-      <c r="AB55" s="99" t="s">
+      <c r="AB55" s="100" t="s">
         <v>200</v>
       </c>
-      <c r="AC55" s="102" t="s">
+      <c r="AC55" s="103" t="s">
         <v>212</v>
       </c>
       <c r="AD55" s="1"/>
@@ -6957,8 +7146,8 @@
       <c r="AA56" s="84" t="s">
         <v>190</v>
       </c>
-      <c r="AB56" s="100"/>
-      <c r="AC56" s="103"/>
+      <c r="AB56" s="101"/>
+      <c r="AC56" s="104"/>
       <c r="AD56" s="1"/>
       <c r="AE56" s="1"/>
       <c r="AF56" s="1"/>
@@ -7032,8 +7221,8 @@
       <c r="Y57" s="1"/>
       <c r="Z57" s="85"/>
       <c r="AA57" s="86"/>
-      <c r="AB57" s="101"/>
-      <c r="AC57" s="104"/>
+      <c r="AB57" s="102"/>
+      <c r="AC57" s="105"/>
       <c r="AD57" s="1"/>
       <c r="AE57" s="1"/>
       <c r="AF57" s="1"/>
@@ -7106,15 +7295,15 @@
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
       <c r="Z58" s="75" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AA58" s="80" t="s">
         <v>191</v>
       </c>
-      <c r="AB58" s="106" t="s">
+      <c r="AB58" s="96" t="s">
         <v>201</v>
       </c>
-      <c r="AC58" s="107" t="s">
+      <c r="AC58" s="98" t="s">
         <v>213</v>
       </c>
       <c r="AD58" s="1"/>
@@ -7194,8 +7383,8 @@
       <c r="AA59" s="78" t="s">
         <v>190</v>
       </c>
-      <c r="AB59" s="92"/>
-      <c r="AC59" s="94"/>
+      <c r="AB59" s="89"/>
+      <c r="AC59" s="91"/>
       <c r="AD59" s="1"/>
       <c r="AE59" s="1"/>
       <c r="AF59" s="1"/>
@@ -7269,8 +7458,8 @@
       <c r="Y60" s="1"/>
       <c r="Z60" s="77"/>
       <c r="AA60" s="79"/>
-      <c r="AB60" s="93"/>
-      <c r="AC60" s="95"/>
+      <c r="AB60" s="97"/>
+      <c r="AC60" s="99"/>
       <c r="AD60" s="1"/>
       <c r="AE60" s="1"/>
       <c r="AF60" s="1"/>
@@ -7343,15 +7532,15 @@
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="83" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="AA61" s="82" t="s">
         <v>187</v>
       </c>
-      <c r="AB61" s="99" t="s">
+      <c r="AB61" s="100" t="s">
         <v>202</v>
       </c>
-      <c r="AC61" s="102" t="s">
+      <c r="AC61" s="103" t="s">
         <v>212</v>
       </c>
       <c r="AD61" s="1"/>
@@ -7431,8 +7620,8 @@
       <c r="AA62" s="84" t="s">
         <v>190</v>
       </c>
-      <c r="AB62" s="100"/>
-      <c r="AC62" s="103"/>
+      <c r="AB62" s="101"/>
+      <c r="AC62" s="104"/>
       <c r="AD62" s="1"/>
       <c r="AE62" s="1"/>
       <c r="AF62" s="1"/>
@@ -7506,8 +7695,8 @@
       <c r="Y63" s="1"/>
       <c r="Z63" s="85"/>
       <c r="AA63" s="86"/>
-      <c r="AB63" s="101"/>
-      <c r="AC63" s="104"/>
+      <c r="AB63" s="102"/>
+      <c r="AC63" s="105"/>
       <c r="AD63" s="1"/>
       <c r="AE63" s="1"/>
       <c r="AF63" s="1"/>
@@ -7580,15 +7769,15 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="1"/>
       <c r="Z64" s="75" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="AA64" s="78" t="s">
         <v>188</v>
       </c>
-      <c r="AB64" s="92" t="s">
+      <c r="AB64" s="89" t="s">
         <v>203</v>
       </c>
-      <c r="AC64" s="94" t="s">
+      <c r="AC64" s="91" t="s">
         <v>213</v>
       </c>
       <c r="AD64" s="1"/>
@@ -7668,8 +7857,8 @@
       <c r="AA65" s="78" t="s">
         <v>190</v>
       </c>
-      <c r="AB65" s="92"/>
-      <c r="AC65" s="94"/>
+      <c r="AB65" s="89"/>
+      <c r="AC65" s="91"/>
       <c r="AD65" s="1"/>
       <c r="AE65" s="1"/>
       <c r="AF65" s="1"/>
@@ -7743,8 +7932,8 @@
       <c r="Y66" s="1"/>
       <c r="Z66" s="76"/>
       <c r="AA66" s="81"/>
-      <c r="AB66" s="108"/>
-      <c r="AC66" s="109"/>
+      <c r="AB66" s="90"/>
+      <c r="AC66" s="92"/>
       <c r="AD66" s="1"/>
       <c r="AE66" s="1"/>
       <c r="AF66" s="1"/>
@@ -7969,7 +8158,7 @@
       <c r="X69" s="1"/>
       <c r="Y69" s="1"/>
       <c r="Z69" s="1" t="s">
-        <v>227</v>
+        <v>257</v>
       </c>
       <c r="AA69" s="1"/>
       <c r="AB69" s="1"/>
@@ -8046,7 +8235,7 @@
       <c r="X70" s="1"/>
       <c r="Y70" s="1"/>
       <c r="Z70" s="1" t="s">
-        <v>228</v>
+        <v>258</v>
       </c>
       <c r="AA70" s="1"/>
       <c r="AB70" s="1"/>
@@ -38503,6 +38692,35 @@
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="R4:Y4"/>
+    <mergeCell ref="Z16:Z18"/>
+    <mergeCell ref="AB16:AB18"/>
+    <mergeCell ref="AC16:AC18"/>
+    <mergeCell ref="Z19:Z21"/>
+    <mergeCell ref="AB19:AB21"/>
+    <mergeCell ref="AC19:AC21"/>
+    <mergeCell ref="Z25:Z27"/>
+    <mergeCell ref="AB25:AB27"/>
+    <mergeCell ref="AC25:AC27"/>
+    <mergeCell ref="Z28:Z30"/>
+    <mergeCell ref="AB28:AB30"/>
+    <mergeCell ref="AC28:AC30"/>
+    <mergeCell ref="Z31:Z33"/>
+    <mergeCell ref="AB31:AB33"/>
+    <mergeCell ref="AC31:AC33"/>
+    <mergeCell ref="Z34:Z36"/>
+    <mergeCell ref="AB34:AB36"/>
+    <mergeCell ref="AC34:AC36"/>
+    <mergeCell ref="Z37:Z39"/>
+    <mergeCell ref="AB37:AB39"/>
+    <mergeCell ref="AC37:AC39"/>
+    <mergeCell ref="AC52:AC54"/>
+    <mergeCell ref="Z40:Z42"/>
+    <mergeCell ref="AB40:AB42"/>
+    <mergeCell ref="AC40:AC42"/>
+    <mergeCell ref="AB43:AB45"/>
+    <mergeCell ref="AC43:AC45"/>
     <mergeCell ref="AB64:AB66"/>
     <mergeCell ref="AC64:AC66"/>
     <mergeCell ref="Z22:Z24"/>
@@ -38519,35 +38737,6 @@
     <mergeCell ref="AB49:AB51"/>
     <mergeCell ref="AC49:AC51"/>
     <mergeCell ref="AB52:AB54"/>
-    <mergeCell ref="AC52:AC54"/>
-    <mergeCell ref="Z40:Z42"/>
-    <mergeCell ref="AB40:AB42"/>
-    <mergeCell ref="AC40:AC42"/>
-    <mergeCell ref="AB43:AB45"/>
-    <mergeCell ref="AC43:AC45"/>
-    <mergeCell ref="Z34:Z36"/>
-    <mergeCell ref="AB34:AB36"/>
-    <mergeCell ref="AC34:AC36"/>
-    <mergeCell ref="Z37:Z39"/>
-    <mergeCell ref="AB37:AB39"/>
-    <mergeCell ref="AC37:AC39"/>
-    <mergeCell ref="Z28:Z30"/>
-    <mergeCell ref="AB28:AB30"/>
-    <mergeCell ref="AC28:AC30"/>
-    <mergeCell ref="Z31:Z33"/>
-    <mergeCell ref="AB31:AB33"/>
-    <mergeCell ref="AC31:AC33"/>
-    <mergeCell ref="Z19:Z21"/>
-    <mergeCell ref="AB19:AB21"/>
-    <mergeCell ref="AC19:AC21"/>
-    <mergeCell ref="Z25:Z27"/>
-    <mergeCell ref="AB25:AB27"/>
-    <mergeCell ref="AC25:AC27"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="R4:Y4"/>
-    <mergeCell ref="Z16:Z18"/>
-    <mergeCell ref="AB16:AB18"/>
-    <mergeCell ref="AC16:AC18"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>